<commit_message>
Update Toto Predictor Lite Draw 616226
</commit_message>
<xml_diff>
--- a/TotoHistoryAll.xlsx
+++ b/TotoHistoryAll.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5663"/>
+  <dimension ref="A1:E5664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -96709,6 +96709,23 @@
         <v>5661</v>
       </c>
     </row>
+    <row r="5664">
+      <c r="A5664" t="n">
+        <v>616226</v>
+      </c>
+      <c r="B5664" t="n">
+        <v>20260726</v>
+      </c>
+      <c r="C5664" t="n">
+        <v>7338</v>
+      </c>
+      <c r="D5664" t="n">
+        <v>9053</v>
+      </c>
+      <c r="E5664" t="n">
+        <v>6235</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Toto Predictor Lite Draw 616326
</commit_message>
<xml_diff>
--- a/TotoHistoryAll.xlsx
+++ b/TotoHistoryAll.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5664"/>
+  <dimension ref="A1:E5665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -96726,6 +96726,23 @@
         <v>6235</v>
       </c>
     </row>
+    <row r="5665">
+      <c r="A5665" t="n">
+        <v>616326</v>
+      </c>
+      <c r="B5665" t="n">
+        <v>20260728</v>
+      </c>
+      <c r="C5665" t="n">
+        <v>1131</v>
+      </c>
+      <c r="D5665" t="n">
+        <v>3649</v>
+      </c>
+      <c r="E5665" t="n">
+        <v>5515</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Toto Predictor Lite Draw 616426
</commit_message>
<xml_diff>
--- a/TotoHistoryAll.xlsx
+++ b/TotoHistoryAll.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5665"/>
+  <dimension ref="A1:E5666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -96743,6 +96743,23 @@
         <v>5515</v>
       </c>
     </row>
+    <row r="5666">
+      <c r="A5666" t="n">
+        <v>616426</v>
+      </c>
+      <c r="B5666" t="n">
+        <v>20260729</v>
+      </c>
+      <c r="C5666" t="n">
+        <v>6225</v>
+      </c>
+      <c r="D5666" t="n">
+        <v>4030</v>
+      </c>
+      <c r="E5666" t="n">
+        <v>8017</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>